<commit_message>
update food ordering app
</commit_message>
<xml_diff>
--- a/food-ordering/backend/uploads/admin_revenue/revenue.xlsx
+++ b/food-ordering/backend/uploads/admin_revenue/revenue.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Month</t>
   </si>
@@ -25,10 +25,16 @@
     <t>Created At</t>
   </si>
   <si>
-    <t>2025-11</t>
-  </si>
-  <si>
-    <t>2025-11-22</t>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2025-12-01</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-06-06</t>
   </si>
 </sst>
 </file>
@@ -405,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="20" customWidth="1"/>
@@ -430,13 +436,27 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>4158</v>
+        <v>1434.3</v>
       </c>
       <c r="C2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>543.9</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>